<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.001-04 Le tunnel du drap
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.001-04.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.001-04.xlsx
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut un tunnel pour la voiture de bois. Le cerceau roule dans les feuilles. Aniss est plus petit. Ils tiennent drap et cerceau plus bas. La voiture passe.</t>
+          <t>Le fil à linge fait tic dans la cour. Une feuille colle au cerceau rouge. Sur le fer, un éclat de cerceau brille. Nina veut un tunnel pour la voiture, maintenant. Elle saisit trop vite : le cerceau roule. Aniss arrive. Elle invite, il attend, ils tiennent le fer. Le drap glisse. Elle refuse de foncer. Merci vécu. L'éclat de cerceau tient sur le fer.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le drap blanc sent le soleil. Il a séché sur le fil. Une pince à linge tient un coin. Le cerceau rouge est contre le mur. Une petite voiture de bois attend. Ses roues sont un peu poussiéreuses. Tu as senti le drap, Nina ? Oui, papa. Il est chaud. Oui. Je veux un tunnel pour la voiture. Avec le cerceau et le drap ? Oui. En ce moment, Nina prend le cerceau. Le fer est tiède. Il fait un petit ding contre le mur. Aniss arrive près du fil. Aniss est plus petit. Nina est plus grande. Ils ont des tailles différentes. Tu viens ? On fait un tunnel. Oui. Nina tient le cerceau debout. Le cerceau part, tout seul. Il roule dans les feuilles sèches. Il est parti ! On le reprend ensemble. Aniss ramène le bas. Nina ramène le haut. Les feuilles raclent le fer. Il fait ding ! Oui. Vous jouez ensemble. On peut jouer ensemble. Nina veut tenir le cerceau haut. Aniss n'atteint pas le haut. Le haut est loin. On le pose plus bas, alors. Le cerceau repose sur l'herbe. Aniss tient un coin du drap. Nina tient l'autre coin. Le tunnel est prêt ? Presque.</t>
+          <t>Le fil à linge fait tic, dans la cour. Le tic est sec, un peu vif. La chaleur pique les pieds nus. Un drap blanc pend au soleil. Le tissu est chaud, un peu rêche. Il sent le soleil, papa. Tu as mis la main dessus ? Oui, papa. C'est chaud. Le drap a séché sur le fil. Une feuille sèche colle au cerceau rouge. Le cerceau rouge attend contre le mur. Nina lève la feuille du fer. Sur le fer, un éclat de cerceau brille. Il brille, maman ! Tu le vois, sur le fer ? Oui, il brille. Une petite voiture de bois attend à l'ombre. Ses roues sont un peu poussiéreuses. Je veux un tunnel, maintenant ! Pour la voiture ? Oui, avec le cerceau. Avec le drap aussi ? Oui, maman. Nina saisit le cerceau trop vite. Le fer glisse entre ses doigts. Le cerceau roule dans les feuilles sèches. Il est parti ! L'éclat de cerceau tremble, puis tient. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu, lourdes. Papa s'accroupit à la même hauteur. Tu veux le tunnel avec Aniss ? Oui, papa. Tes pieds sont dans l'herbe ? Oui, maman. En ce moment, Aniss arrive près du fil. Il a les genoux un peu verts. Tu viens ? On fait un tunnel. Aniss ne dit rien, d'abord. Il regarde le cerceau, puis Nina. Oui. Nina veut tenir le cerceau bien haut. Aniss tend les mains, trop bas. Les doigts d'Aniss glissent sur le fer. Le haut est loin. Attends. Nina baisse un peu les bras. Aniss tient le bas du cerceau. Nina tient le haut, moins loin. Vous tenez le fer ? Oui, papa. Moi, le bas.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le drap blanc sent le soleil. Il a séché sur le fil. Une pince à linge tient un coin. Le cerceau rouge est contre le mur. Une petite voiture de bois attend. Ses roues sont un peu poussiéreuses. Tu as senti le drap, Nina ? Oui, papa. Il est chaud. Oui. Je veux un tunnel pour la voiture. Avec le cerceau et le drap ? Oui. En ce moment, Nina prend le cerceau. Le fer est tiède. Il fait un petit ding contre le mur. Aniss arrive près du fil. Aniss est plus petit. Nina est plus grande. Ils ont des tailles différentes. Tu viens ? On fait un tunnel. Oui. Nina tient le cerceau debout. Le cerceau part, tout seul. Il roule dans les feuilles sèches. Il est parti ! On le reprend ensemble. Aniss ramène le bas. Nina ramène le haut. Les feuilles raclent le fer. Il fait ding ! Oui. Vous jouez ensemble. On peut jouer ensemble. Nina veut tenir le cerceau haut. Aniss n'atteint pas le haut. Le haut est loin. On le pose plus bas, alors. Le cerceau repose sur l'herbe. Aniss tient un coin du drap. Nina tient l'autre coin. Le tunnel est prêt ? Presque.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le fil à linge fait tic, dans la cour. Le tic est sec, un peu vif. La chaleur pique les pieds nus. Un drap blanc pend au soleil. Le tissu est chaud, un peu rêche. Il sent le soleil, papa. Tu as mis la main dessus ? Oui, papa. C'est chaud. Le drap a séché sur le fil. Une feuille sèche colle au cerceau rouge. Le cerceau rouge attend contre le mur. Nina lève la feuille du fer. Sur le fer, un &lt;emphasis level="moderate"&gt;éclat de cerceau&lt;/emphasis&gt; brille. Il brille, maman ! Tu le vois, sur le fer ? Oui, il brille. Une petite voiture de bois attend à l'ombre. Ses roues sont un peu poussiéreuses. Je veux un tunnel, maintenant ! Pour la voiture ? Oui, avec le cerceau. Avec le drap aussi ? Oui, maman. Nina saisit le cerceau trop vite. Le fer glisse entre ses doigts. Le cerceau roule dans les feuilles sèches. Il est parti ! L'éclat de cerceau tremble, puis tient. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu, lourdes. Papa s'accroupit à la même hauteur. Tu veux le tunnel avec Aniss ? Oui, papa. Tes pieds sont dans l'herbe ? Oui, maman. En ce moment, Aniss arrive près du fil. Il a les genoux un peu verts. Tu viens ? On fait un tunnel. Aniss ne dit rien, d'abord. Il regarde le cerceau, puis Nina. Oui. Nina veut tenir le cerceau bien haut. Aniss tend les mains, trop bas. Les doigts d'Aniss glissent sur le fer. Le haut est loin. Attends. Nina baisse un peu les bras. Aniss tient le bas du cerceau. Nina tient le haut, moins loin. Vous tenez le fer ? Oui, papa. Moi, le bas.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Kamil arrive au parc. Papa s'assoit sur le banc. Ava arrive avec un cerceau. Ava est plus petite que Kamil. Kamil est plus grand qu'Ava. Ils ont des &lt;emphasis&gt;tailles&lt;/emphasis&gt; différentes. Kamil l'invite. Il dit : viens jouer. Ava dit : oui. Ils jouent ensemble près du cerceau. Kamil tient un bout. Ava tient l'autre bout. Les tailles différentes restent là. Ils font rouler le cerceau. Papa dit : vous jouez ensemble. Plus tard, ils rentrent. Maman pose un tapis. Sami est là. Sami est plus petit que Kamil. Encore des tailles différentes. Kamil invite Sami. Ils jouent ensemble avec les cubes. Kamil pose un cube. Sami pose un cube. Au parc, puis au salon, c'est pareil. On invite. On joue ensemble. Petit ou grand, on joue ensemble. Maman dit : vous avez des tailles différentes. Et vous jouez ensemble. [pause]</t>
+          <t>Le fil à linge fait tic, dans la cour. Le tic est sec, un peu vif. La chaleur pique les pieds nus. Un drap blanc pend au soleil. Le tissu est chaud, un peu rêche. Il sent le soleil, papa. Tu as mis la main dessus ? Oui, papa. C'est chaud. Le drap a séché sur le fil. Une feuille sèche colle au cerceau rouge. Le cerceau rouge attend contre le mur. Nina lève la feuille du fer. Sur le fer, un &lt;emphasis&gt;éclat de cerceau&lt;/emphasis&gt; brille. Il brille, maman ! Tu le vois, sur le fer ? Oui, il brille. Une petite voiture de bois attend à l'ombre. Ses roues sont un peu poussiéreuses. Je veux un tunnel, maintenant ! Pour la voiture ? Oui, avec le cerceau. Avec le drap aussi ? Oui, maman. Nina saisit le cerceau trop vite. Le fer glisse entre ses doigts. Le cerceau roule dans les feuilles sèches. Il est parti ! L'éclat de cerceau tremble, puis tient. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu, lourdes. Papa s'accroupit à la même hauteur. Tu veux le tunnel avec Aniss ? Oui, papa. Tes pieds sont dans l'herbe ? Oui, maman. En ce moment, Aniss arrive près du fil. Il a les genoux un peu verts. Tu viens ? On fait un tunnel. Aniss ne dit rien, d'abord. Il regarde le cerceau, puis Nina. Oui. Nina veut tenir le cerceau bien haut. Aniss tend les mains, trop bas. Les doigts d'Aniss glissent sur le fer. Le haut est loin. Attends. Nina baisse un peu les bras. Aniss tient le bas du cerceau. Nina tient le haut, moins loin. Vous tenez le fer ? Oui, papa. Moi, le bas. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>tailles</t>
+          <t>éclat de cerceau</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,53 +1326,68 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_tunnel_avec_aniss_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le drap blanc sent le soleil.
-narrateur|Il a séché sur le fil.
-narrateur|Une pince à linge tient un coin.
-narrateur|Le cerceau rouge est contre le mur.
-narrateur|Une petite voiture de bois attend.
+          <t>narrateur|Le fil à linge fait tic, dans la cour.
+narrateur|Le tic est sec, un peu vif.
+narrateur|La chaleur pique les pieds nus.
+narrateur|Un drap blanc pend au soleil.
+narrateur|Le tissu est chaud, un peu rêche.
+enfant-f|Il sent le soleil, papa.
+papa|Tu as mis la main dessus ?
+enfant-f|Oui, papa.
+enfant-f|C'est chaud.
+maman|Le drap a séché sur le fil.
+narrateur|Une feuille sèche colle au cerceau rouge.
+narrateur|Le cerceau rouge attend contre le mur.
+narrateur|Nina lève la feuille du fer.
+narrateur|Sur le fer, un éclat de cerceau brille.
+enfant-f|Il brille, maman !
+maman|Tu le vois, sur le fer ?
+enfant-f|Oui, il brille.
+narrateur|Une petite voiture de bois attend à l'ombre.
 narrateur|Ses roues sont un peu poussiéreuses.
-papa|Tu as senti le drap, Nina ?
+enfant-f|Je veux un tunnel, maintenant !
+papa|Pour la voiture ?
+enfant-f|Oui, avec le cerceau.
+maman|Avec le drap aussi ?
+enfant-f|Oui, maman.
+narrateur|Nina saisit le cerceau trop vite.
+narrateur|Le fer glisse entre ses doigts.
+narrateur|Le cerceau roule dans les feuilles sèches.
+enfant-f|Il est parti !
+narrateur|L'éclat de cerceau tremble, puis tient.
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu, lourdes.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu veux le tunnel avec Aniss ?
 enfant-f|Oui, papa.
-enfant-f|Il est chaud.
-papa|Oui.
-enfant-f|Je veux un tunnel pour la voiture.
-maman|Avec le cerceau et le drap ?
-enfant-f|Oui.
-narrateur|En ce moment, Nina prend le cerceau.
-narrateur|Le fer est tiède.
-narrateur|Il fait un petit ding contre le mur.
-narrateur|Aniss arrive près du fil.
-narrateur|Aniss est plus petit.
-narrateur|Nina est plus grande.
-narrateur|Ils ont des tailles différentes.
+maman|Tes pieds sont dans l'herbe ?
+enfant-f|Oui, maman.
+narrateur|En ce moment, Aniss arrive près du fil.
+narrateur|Il a les genoux un peu verts.
 enfant-f|Tu viens ?
 enfant-f|On fait un tunnel.
+narrateur|Aniss ne dit rien, d'abord.
+narrateur|Il regarde le cerceau, puis Nina.
 copain|Oui.
-narrateur|Nina tient le cerceau debout.
-narrateur|Le cerceau part, tout seul.
-narrateur|Il roule dans les feuilles sèches.
-enfant-f|Il est parti !
-papa|On le reprend ensemble.
-narrateur|Aniss ramène le bas.
-narrateur|Nina ramène le haut.
-narrateur|Les feuilles raclent le fer.
-copain|Il fait ding !
-papa|Oui.
-maman|Vous jouez ensemble.
-maman|On peut jouer ensemble.
-narrateur|Nina veut tenir le cerceau haut.
-narrateur|Aniss n'atteint pas le haut.
+narrateur|Nina veut tenir le cerceau bien haut.
+narrateur|Aniss tend les mains, trop bas.
+narrateur|Les doigts d'Aniss glissent sur le fer.
 enfant-f|Le haut est loin.
-maman|On le pose plus bas, alors.
-narrateur|Le cerceau repose sur l'herbe.
-narrateur|Aniss tient un coin du drap.
-narrateur|Nina tient l'autre coin.
-papa|Le tunnel est prêt ?
-enfant-f|Presque.</t>
+copain|Attends.
+narrateur|Nina baisse un peu les bras.
+narrateur|Aniss tient le bas du cerceau.
+narrateur|Nina tient le haut, moins loin.
+papa|Vous tenez le fer ?
+enfant-f|Oui, papa.
+copain|Moi, le bas.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1409,12 +1424,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nina invite Aniss. Que font-ils ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina invite &lt;emphasis level="moderate"&gt;Aniss&lt;/emphasis&gt;. Que font-ils ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Kamil invite Ava, puis Sami. Que font-ils ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nina invite &lt;emphasis&gt;Aniss&lt;/emphasis&gt;. Que font-ils ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1477,7 +1492,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1485,10 +1500,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1503,34 +1518,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Aniss</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1539,23 +1558,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=nina_invite_ils_tiennent_le_fer_ensemble; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1588,17 +1607,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Le drap tombe sur le cerceau. Ça fait une petite grotte claire. La lumière passe à travers. C'est blanc, dedans. Oui. Nina pousse la voiture. Aniss l'attend de l'autre côté. Les roues font un bruit de bois. Elle arrive ! Elle est passée. Les deux façons marchent. Vous avez des tailles différentes. Et vous jouez ensemble. Encore un tour ? Oui, papa. Aniss pousse, cette fois. Nina attend, tout bas. La voiture ressort, un peu chaude. Une feuille sèche est restée dessus. Elle vient du platane, ça. Oui. Le fil à linge claque un peu. La pince tient encore le coin. Le tunnel tient bien ? Oui, maman.</t>
+          <t>Le drap tombe sur le cerceau. Ça fait une petite grotte claire. La lumière passe à travers le tissu. C'est blanc, dedans. Oui. Nina pousse la voiture trop vite. Le drap glisse d'un côté. Les roues s'arrêtent dans le tissu. Elle ne passe pas. Le sourire de Nina ne revient pas. Nina refuse de foncer, cette fois. Elle pose les mains sur le drap. Personne ne dit la suite à voix haute. Elle regarde le cerceau, elle écoute la cour. Le fil à linge fait tic, sec. Sur le fer, l'éclat de cerceau brille. Tu tiens ce coin ? Aniss ne dit rien. Il pose une main sur le drap, sans parler. Oui. Nina attend que la grotte tienne. Elle pousse la voiture, sans se presser. Les roues font un bruit de bois. Elle arrive ! Elle est passée. Merci, Nina. Papa a vu les deux mains sur le drap. Aniss, tu as vu la voiture ? Oui. Un autre tour ? Oui, papa. Aniss pousse, à son tour. Nina attend de l'autre côté. La voiture ressort, un peu chaude. Une feuille sèche est restée dessus. Elle vient du platane, ça ? Oui. Le ventre de Nina se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Le drap tombe sur le cerceau. Ça fait une petite grotte claire. La lumière passe à travers. C'est blanc, dedans. Oui. Nina pousse la voiture. Aniss l'attend de l'autre côté. Les roues font un bruit de bois. Elle arrive ! Elle est passée. Les deux façons marchent. Vous avez des tailles différentes. Et vous jouez ensemble. Encore un tour ? Oui, papa. Aniss pousse, cette fois. Nina attend, tout bas. La voiture ressort, un peu chaude. Une feuille sèche est restée dessus. Elle vient du platane, ça. Oui. Le fil à linge claque un peu. La pince tient encore le coin. Le tunnel tient bien ? Oui, maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;drap&lt;/emphasis&gt; tombe sur le cerceau. Ça fait une petite grotte claire. La lumière passe à travers le tissu. C'est blanc, dedans. Oui. Nina pousse la voiture trop vite. Le drap glisse d'un côté. Les roues s'arrêtent dans le tissu. Elle ne passe pas. Le sourire de Nina ne revient pas. Nina refuse de foncer, cette fois. Elle pose les mains sur le drap. Personne ne dit la suite à voix haute. Elle regarde le cerceau, elle écoute la cour. Le fil à linge fait tic, sec. Sur le fer, l'éclat de cerceau brille. Tu tiens ce coin ? Aniss ne dit rien. Il pose une main sur le drap, sans parler. Oui. Nina attend que la grotte tienne. Elle pousse la voiture, sans se presser. Les roues font un bruit de bois. Elle arrive ! Elle est passée. Merci, Nina. Papa a vu les deux mains sur le drap. Aniss, tu as vu la voiture ? Oui. Un autre tour ? Oui, papa. Aniss pousse, à son tour. Nina attend de l'autre côté. La voiture ressort, un peu chaude. Une feuille sèche est restée dessus. Elle vient du platane, ça ? Oui. Le ventre de Nina se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Kamil a invité. Ils ont des &lt;emphasis&gt;tailles&lt;/emphasis&gt; différentes. Ils jouent ensemble. [pause]</t>
+          <t>Le &lt;emphasis&gt;drap&lt;/emphasis&gt; tombe sur le cerceau. Ça fait une petite grotte claire. La lumière passe à travers le tissu. C'est blanc, dedans. Oui. Nina pousse la voiture trop vite. Le drap glisse d'un côté. Les roues s'arrêtent dans le tissu. Elle ne passe pas. Le sourire de Nina ne revient pas. Nina refuse de foncer, cette fois. Elle pose les mains sur le drap. Personne ne dit la suite à voix haute. Elle regarde le cerceau, elle écoute la cour. Le fil à linge fait tic, sec. Sur le fer, l'éclat de cerceau brille. Tu tiens ce coin ? Aniss ne dit rien. Il pose une main sur le drap, sans parler. Oui. Nina attend que la grotte tienne. Elle pousse la voiture, sans se presser. Les roues font un bruit de bois. Elle arrive ! Elle est passée. Merci, Nina. Papa a vu les deux mains sur le drap. Aniss, tu as vu la voiture ? Oui. Un autre tour ? Oui, papa. Aniss pousse, à son tour. Nina attend de l'autre côté. La voiture ressort, un peu chaude. Une feuille sèche est restée dessus. Elle vient du platane, ça ? Oui. Le ventre de Nina se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1645,7 +1664,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1653,10 +1672,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1679,30 +1698,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>tailles</t>
+          <t>drap</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1711,10 +1730,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1727,36 +1746,54 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_attend_aniss_tient_le_drap; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
           <t>narrateur|Le drap tombe sur le cerceau.
 narrateur|Ça fait une petite grotte claire.
-narrateur|La lumière passe à travers.
+narrateur|La lumière passe à travers le tissu.
 enfant-f|C'est blanc, dedans.
 papa|Oui.
-narrateur|Nina pousse la voiture.
-narrateur|Aniss l'attend de l'autre côté.
+narrateur|Nina pousse la voiture trop vite.
+narrateur|Le drap glisse d'un côté.
+narrateur|Les roues s'arrêtent dans le tissu.
+enfant-f|Elle ne passe pas.
+narrateur|Le sourire de Nina ne revient pas.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Elle pose les mains sur le drap.
+narrateur|Personne ne dit la suite à voix haute.
+narrateur|Elle regarde le cerceau, elle écoute la cour.
+narrateur|Le fil à linge fait tic, sec.
+narrateur|Sur le fer, l'éclat de cerceau brille.
+enfant-f|Tu tiens ce coin ?
+narrateur|Aniss ne dit rien.
+narrateur|Il pose une main sur le drap, sans parler.
+copain|Oui.
+narrateur|Nina attend que la grotte tienne.
+narrateur|Elle pousse la voiture, sans se presser.
 narrateur|Les roues font un bruit de bois.
 copain|Elle arrive !
 enfant-f|Elle est passée.
-maman|Les deux façons marchent.
-maman|Vous avez des tailles différentes.
-maman|Et vous jouez ensemble.
-papa|Encore un tour ?
+papa|Merci, Nina.
+narrateur|Papa a vu les deux mains sur le drap.
+maman|Aniss, tu as vu la voiture ?
+copain|Oui.
+papa|Un autre tour ?
 enfant-f|Oui, papa.
-narrateur|Aniss pousse, cette fois.
-narrateur|Nina attend, tout bas.
+narrateur|Aniss pousse, à son tour.
+narrateur|Nina attend de l'autre côté.
 narrateur|La voiture ressort, un peu chaude.
 narrateur|Une feuille sèche est restée dessus.
-papa|Elle vient du platane, ça.
+papa|Elle vient du platane, ça ?
 enfant-f|Oui.
-narrateur|Le fil à linge claque un peu.
-narrateur|La pince tient encore le coin.
-maman|Le tunnel tient bien ?
-enfant-f|Oui, maman.</t>
+narrateur|Le ventre de Nina se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>drap,voiture</t>
         </is>
       </c>
     </row>
@@ -1783,17 +1820,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On plie le drap ? Oui. Nina plie le drap, tout doux. Aniss pose le cerceau contre le mur. La voiture rentre dans une chaussure. Tu as fini de plier le drap ? Oui, papa. À demain. À demain. Le fil à linge redevient calme. Les feuilles sèches ne bougent plus. On se lave les mains ? Oui.</t>
+          <t>Nina veut le cerceau plus haut, d'un coup. Elle lève le fer trop vite. Aniss n'atteint plus le bas. Attends. Je le tiens ! Le cerceau penche vers l'herbe. Le drap glisse, presque. Ça tombe ! Nina veut rattraper le fer, d'un coup. Nina refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde le cerceau. Elle écoute le tic du fil. Le fer est tiède sous les doigts. L'éclat, papa ? Tu le vois, toi ? Non, plus sur le fer. Nina baisse le cerceau, sans se presser. Aniss reprend le bas. Il est là. Sur ce fer ? Oui, sur ce fer. L'éclat de cerceau revient, sur le fer. La voiture, Nina ? Oui. Ils tiennent le drap, l'un et l'autre. La voiture traverse la grotte claire. C'est passé. Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On plie le drap ? Oui. Nina plie le drap, tout doux. Aniss pose le cerceau contre le mur. La voiture rentre dans une chaussure. Tu as fini de plier le drap ? Oui, papa. À demain. À demain. Le fil à linge redevient calme. Les feuilles sèches ne bougent plus. On se lave les mains ? Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina veut le cerceau plus haut, d'un coup. Elle lève le fer trop vite. Aniss n'atteint plus le bas. Attends. Je le tiens ! Le cerceau penche vers l'herbe. Le drap glisse, presque. Ça tombe ! Nina veut rattraper le fer, d'un coup. Nina refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde le cerceau. Elle écoute le tic du fil. Le fer est tiède sous les doigts. L'éclat, papa ? Tu le vois, toi ? Non, plus sur le fer. Nina baisse le cerceau, sans se presser. Aniss reprend le bas. Il est là. Sur ce fer ? Oui, sur ce fer. L'&lt;emphasis level="moderate"&gt;éclat de cerceau&lt;/emphasis&gt; revient, sur le fer. La voiture, Nina ? Oui. Ils tiennent le drap, l'un et l'autre. La voiture traverse la grotte claire. C'est passé. Oui.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Kamil range un cube. Ava range le cerceau. [pause]</t>
+          <t>&lt;low-pitch&gt;Nina veut le cerceau plus haut, d'un coup. Elle lève le fer trop vite. Aniss n'atteint plus le bas. Attends. Je le tiens ! Le cerceau penche vers l'herbe. Le drap glisse, presque. Ça tombe ! Nina veut rattraper le fer, d'un coup. Nina refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde le cerceau. Elle écoute le tic du fil. Le fer est tiède sous les doigts. L'éclat, papa ? Tu le vois, toi ? Non, plus sur le fer. Nina baisse le cerceau, sans se presser. Aniss reprend le bas. Il est là. Sur ce fer ? Oui, sur ce fer. L'&lt;emphasis&gt;éclat de cerceau&lt;/emphasis&gt; revient, sur le fer. La voiture, Nina ? Oui. Ils tiennent le drap, l'un et l'autre. La voiture traverse la grotte claire. C'est passé. Oui.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1840,7 +1877,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1848,22 +1885,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1872,28 +1913,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cerceau</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1902,36 +1947,63 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|On plie le drap ?
+          <t>narrateur|Nina veut le cerceau plus haut, d'un coup.
+narrateur|Elle lève le fer trop vite.
+narrateur|Aniss n'atteint plus le bas.
+copain|Attends.
+enfant-f|Je le tiens !
+narrateur|Le cerceau penche vers l'herbe.
+narrateur|Le drap glisse, presque.
+enfant-f|Ça tombe !
+narrateur|Nina veut rattraper le fer, d'un coup.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape fort, dans sa poitrine.
+narrateur|Personne ne dit la suite à voix haute.
+narrateur|Elle regarde le cerceau.
+narrateur|Elle écoute le tic du fil.
+narrateur|Le fer est tiède sous les doigts.
+enfant-f|L'éclat, papa ?
+papa|Tu le vois, toi ?
+enfant-f|Non, plus sur le fer.
+narrateur|Nina baisse le cerceau, sans se presser.
+narrateur|Aniss reprend le bas.
+enfant-f|Il est là.
+papa|Sur ce fer ?
+enfant-f|Oui, sur ce fer.
+narrateur|L'éclat de cerceau revient, sur le fer.
+maman|La voiture, Nina ?
 enfant-f|Oui.
-narrateur|Nina plie le drap, tout doux.
-narrateur|Aniss pose le cerceau contre le mur.
-narrateur|La voiture rentre dans une chaussure.
-papa|Tu as fini de plier le drap ?
-enfant-f|Oui, papa.
-copain|À demain.
-enfant-f|À demain.
-narrateur|Le fil à linge redevient calme.
-narrateur|Les feuilles sèches ne bougent plus.
-maman|On se lave les mains ?
-enfant-f|Oui.</t>
+narrateur|Ils tiennent le drap, l'un et l'autre.
+narrateur|La voiture traverse la grotte claire.
+enfant-f|C'est passé.
+copain|Oui.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>cerceau,feuilles</t>
         </is>
       </c>
     </row>
@@ -1958,17 +2030,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La voiture a traversé le tunnel. On a joué ensemble. Bravo, Nina. Le drap sent encore le soleil.</t>
+          <t>Le cerceau rouge repose contre le mur. Une feuille sèche reste collée au fer. L'éclat est là, papa. Tu le vois sur le fer ? Oui, papa. On est bien, ici. Le drap sent le soleil. Le tissu est chaud, un peu rêche. La voiture a traversé. Elle a traversé, Nina. Oui, maman. Nina pose la joue près du drap. Le drap est tiède, un peu. C'est chaud. Aniss pose la voiture à l'ombre. Les roues ont une trace d'herbe. L'éclat de cerceau tient sur le fer.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La voiture a traversé le tunnel. On a joué ensemble. Bravo, Nina. Le drap sent encore le soleil.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le cerceau rouge repose contre le mur. Une feuille sèche reste collée au fer. L'éclat est là, papa. Tu le vois sur le fer ? Oui, papa. On est bien, ici. Le drap sent le soleil. Le tissu est chaud, un peu rêche. La voiture a traversé. Elle a traversé, Nina. Oui, maman. Nina pose la joue près du drap. Le drap est tiède, un peu. C'est chaud. Aniss pose la voiture à l'ombre. Les roues ont une trace d'herbe. L'&lt;emphasis level="moderate"&gt;éclat de cerceau&lt;/emphasis&gt; tient sur le fer.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le cerceau rouge repose contre le mur. Une feuille sèche reste collée au fer. L'éclat est là, papa. Tu le vois sur le fer ? Oui, papa. On est bien, ici. Le drap sent le soleil. Le tissu est chaud, un peu rêche. La voiture a traversé. Elle a traversé, Nina. Oui, maman. Nina pose la joue près du drap. Le drap est tiède, un peu. C'est chaud. Aniss pose la voiture à l'ombre. Les roues ont une trace d'herbe. L'&lt;emphasis&gt;éclat de cerceau&lt;/emphasis&gt; tient sur le fer.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2015,15 +2087,15 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2035,12 +2107,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2049,17 +2121,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cerceau</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2068,11 +2144,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2081,27 +2157,49 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_fer; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|La voiture a traversé le tunnel.
-enfant-f|On a joué ensemble.
-maman|Bravo, Nina.
-narrateur|Le drap sent encore le soleil.</t>
+          <t>narrateur|Le cerceau rouge repose contre le mur.
+narrateur|Une feuille sèche reste collée au fer.
+enfant-f|L'éclat est là, papa.
+papa|Tu le vois sur le fer ?
+enfant-f|Oui, papa.
+maman|On est bien, ici.
+narrateur|Le drap sent le soleil.
+narrateur|Le tissu est chaud, un peu rêche.
+enfant-f|La voiture a traversé.
+maman|Elle a traversé, Nina.
+enfant-f|Oui, maman.
+narrateur|Nina pose la joue près du drap.
+narrateur|Le drap est tiède, un peu.
+enfant-f|C'est chaud.
+narrateur|Aniss pose la voiture à l'ombre.
+narrateur|Les roues ont une trace d'herbe.
+narrateur|L'éclat de cerceau tient sur le fer.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>drap</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2200,6 +2298,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>